<commit_message>
Add evacuation plans tab with nearest safe place routing.
Includes Safe Places dataset, distance-based matching, map view, and updated sample data with coordinates.
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Flood Alerts" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Volunteers" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Safe Places" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +454,16 @@
           <t>Location</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -486,6 +497,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>45.4772</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-73.60253</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -519,6 +536,12 @@
           <t>Longueuil</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>45.53768</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-73.51206000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,6 +575,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>45.43976</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-73.84738</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -585,6 +614,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>45.55629</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-73.65421000000001</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -618,6 +653,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>45.45827</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-73.62246</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -651,6 +692,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H7" t="n">
+        <v>45.45506</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-73.56229</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -684,6 +731,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H8" t="n">
+        <v>45.55158</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-73.65371</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -717,6 +770,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H9" t="n">
+        <v>45.51085</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-73.57026999999999</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -750,6 +809,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H10" t="n">
+        <v>45.54449</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-73.67921</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -783,6 +848,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H11" t="n">
+        <v>45.60689</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-73.72467</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -816,6 +887,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H12" t="n">
+        <v>45.50368</v>
+      </c>
+      <c r="I12" t="n">
+        <v>-73.70826</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -849,6 +926,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H13" t="n">
+        <v>45.45816</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-73.86588999999999</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -882,6 +965,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H14" t="n">
+        <v>45.60683</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-73.72421</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -915,6 +1004,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H15" t="n">
+        <v>45.53405</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-73.57743000000001</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -948,6 +1043,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H16" t="n">
+        <v>45.45947</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-73.61472000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -981,6 +1082,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H17" t="n">
+        <v>45.53267</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-73.58271000000001</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1014,6 +1121,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H18" t="n">
+        <v>45.45754</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-73.56686999999999</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1047,6 +1160,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H19" t="n">
+        <v>45.47814</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-73.62752999999999</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1080,6 +1199,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H20" t="n">
+        <v>45.51047</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-73.56733</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1113,6 +1238,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H21" t="n">
+        <v>45.49643</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-73.70997</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1146,6 +1277,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H22" t="n">
+        <v>45.46436</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-73.62358999999999</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1179,6 +1316,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H23" t="n">
+        <v>45.50944</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-73.57584</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1212,6 +1355,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H24" t="n">
+        <v>45.49164</v>
+      </c>
+      <c r="I24" t="n">
+        <v>-73.58224</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1245,6 +1394,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H25" t="n">
+        <v>45.54484</v>
+      </c>
+      <c r="I25" t="n">
+        <v>-73.67449999999999</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1278,6 +1433,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H26" t="n">
+        <v>45.53408</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-73.57947</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1311,6 +1472,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H27" t="n">
+        <v>45.4894</v>
+      </c>
+      <c r="I27" t="n">
+        <v>-73.69559</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1344,6 +1511,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H28" t="n">
+        <v>45.44123</v>
+      </c>
+      <c r="I28" t="n">
+        <v>-73.85460999999999</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1377,6 +1550,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H29" t="n">
+        <v>45.50045</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-73.55235</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1410,6 +1589,12 @@
           <t>Longueuil</t>
         </is>
       </c>
+      <c r="H30" t="n">
+        <v>45.52729</v>
+      </c>
+      <c r="I30" t="n">
+        <v>-73.52837</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1443,6 +1628,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H31" t="n">
+        <v>45.48507</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-73.62527</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1476,6 +1667,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H32" t="n">
+        <v>45.51843</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-73.61738</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1509,6 +1706,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H33" t="n">
+        <v>45.61071</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-73.71953999999999</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1542,6 +1745,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H34" t="n">
+        <v>45.60797</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-73.70236</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1575,6 +1784,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H35" t="n">
+        <v>45.4507</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-73.57491</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1608,6 +1823,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H36" t="n">
+        <v>45.62089</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-73.70308</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1641,6 +1862,12 @@
           <t>Hochelaga</t>
         </is>
       </c>
+      <c r="H37" t="n">
+        <v>45.55382</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-73.55</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1674,6 +1901,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H38" t="n">
+        <v>45.55069</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-73.65877999999999</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1707,6 +1940,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H39" t="n">
+        <v>45.44563</v>
+      </c>
+      <c r="I39" t="n">
+        <v>-73.86082</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1740,6 +1979,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H40" t="n">
+        <v>45.43625</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-73.8582</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1773,6 +2018,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H41" t="n">
+        <v>45.50796</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-73.58225</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1806,6 +2057,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H42" t="n">
+        <v>45.52702</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-73.60661</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1839,6 +2096,12 @@
           <t>Hochelaga</t>
         </is>
       </c>
+      <c r="H43" t="n">
+        <v>45.53837</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-73.55418</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1872,6 +2135,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H44" t="n">
+        <v>45.49582</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-73.57599</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1905,6 +2174,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H45" t="n">
+        <v>45.61137</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-73.71889</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1938,6 +2213,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H46" t="n">
+        <v>45.48809</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-73.55278</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1971,6 +2252,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H47" t="n">
+        <v>45.49312</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-73.70262</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2004,6 +2291,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H48" t="n">
+        <v>45.51398</v>
+      </c>
+      <c r="I48" t="n">
+        <v>-73.56995000000001</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2037,6 +2330,12 @@
           <t>Hochelaga</t>
         </is>
       </c>
+      <c r="H49" t="n">
+        <v>45.55626</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-73.54519999999999</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2070,6 +2369,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H50" t="n">
+        <v>45.45807</v>
+      </c>
+      <c r="I50" t="n">
+        <v>-73.86046</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2103,6 +2408,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H51" t="n">
+        <v>45.50892</v>
+      </c>
+      <c r="I51" t="n">
+        <v>-73.59088</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2136,6 +2447,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H52" t="n">
+        <v>45.49291</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-73.5697</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2169,6 +2486,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H53" t="n">
+        <v>45.45336</v>
+      </c>
+      <c r="I53" t="n">
+        <v>-73.5707</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2202,6 +2525,12 @@
           <t>Longueuil</t>
         </is>
       </c>
+      <c r="H54" t="n">
+        <v>45.52439</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-73.51853</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2235,6 +2564,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H55" t="n">
+        <v>45.50731</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-73.58358</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2268,6 +2603,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H56" t="n">
+        <v>45.49562</v>
+      </c>
+      <c r="I56" t="n">
+        <v>-73.70865999999999</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2301,6 +2642,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H57" t="n">
+        <v>45.50806</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-73.56684</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2334,6 +2681,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H58" t="n">
+        <v>45.50534</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-73.57514</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2367,6 +2720,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H59" t="n">
+        <v>45.43322</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-73.62555999999999</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2400,6 +2759,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H60" t="n">
+        <v>45.51404</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-73.71635000000001</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2433,6 +2798,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H61" t="n">
+        <v>45.43848</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-73.63758</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2466,6 +2837,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H62" t="n">
+        <v>45.51462</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-73.70323</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2499,6 +2876,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H63" t="n">
+        <v>45.55415</v>
+      </c>
+      <c r="I63" t="n">
+        <v>-73.65863</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2532,6 +2915,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H64" t="n">
+        <v>45.43505</v>
+      </c>
+      <c r="I64" t="n">
+        <v>-73.63791000000001</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2565,6 +2954,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H65" t="n">
+        <v>45.43604</v>
+      </c>
+      <c r="I65" t="n">
+        <v>-73.63970999999999</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2598,6 +2993,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H66" t="n">
+        <v>45.52076</v>
+      </c>
+      <c r="I66" t="n">
+        <v>-73.61185</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2631,6 +3032,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H67" t="n">
+        <v>45.51681</v>
+      </c>
+      <c r="I67" t="n">
+        <v>-73.5655</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2664,6 +3071,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H68" t="n">
+        <v>45.44799</v>
+      </c>
+      <c r="I68" t="n">
+        <v>-73.56632</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2697,6 +3110,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H69" t="n">
+        <v>45.42349</v>
+      </c>
+      <c r="I69" t="n">
+        <v>-73.64498</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2730,6 +3149,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H70" t="n">
+        <v>45.5033</v>
+      </c>
+      <c r="I70" t="n">
+        <v>-73.56138</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2763,6 +3188,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H71" t="n">
+        <v>45.62056</v>
+      </c>
+      <c r="I71" t="n">
+        <v>-73.71983</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2796,6 +3227,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H72" t="n">
+        <v>45.61593</v>
+      </c>
+      <c r="I72" t="n">
+        <v>-73.69893</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2829,6 +3266,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H73" t="n">
+        <v>45.51791</v>
+      </c>
+      <c r="I73" t="n">
+        <v>-73.56814</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2862,6 +3305,12 @@
           <t>NDG</t>
         </is>
       </c>
+      <c r="H74" t="n">
+        <v>45.48533</v>
+      </c>
+      <c r="I74" t="n">
+        <v>-73.62307</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2895,6 +3344,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H75" t="n">
+        <v>45.56088</v>
+      </c>
+      <c r="I75" t="n">
+        <v>-73.66930000000001</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2928,6 +3383,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H76" t="n">
+        <v>45.45873</v>
+      </c>
+      <c r="I76" t="n">
+        <v>-73.85735</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2961,6 +3422,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H77" t="n">
+        <v>45.59374</v>
+      </c>
+      <c r="I77" t="n">
+        <v>-73.72242</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2994,6 +3461,12 @@
           <t>Plateau</t>
         </is>
       </c>
+      <c r="H78" t="n">
+        <v>45.5227</v>
+      </c>
+      <c r="I78" t="n">
+        <v>-73.58226999999999</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3027,6 +3500,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H79" t="n">
+        <v>45.43261</v>
+      </c>
+      <c r="I79" t="n">
+        <v>-73.64738</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3060,6 +3539,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H80" t="n">
+        <v>45.42808</v>
+      </c>
+      <c r="I80" t="n">
+        <v>-73.62357</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3093,6 +3578,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H81" t="n">
+        <v>45.50661</v>
+      </c>
+      <c r="I81" t="n">
+        <v>-73.71365</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3126,6 +3617,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H82" t="n">
+        <v>45.51175</v>
+      </c>
+      <c r="I82" t="n">
+        <v>-73.69755000000001</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3159,6 +3656,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H83" t="n">
+        <v>45.51266</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-73.62375</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3192,6 +3695,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H84" t="n">
+        <v>45.51767</v>
+      </c>
+      <c r="I84" t="n">
+        <v>-73.61812</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3225,6 +3734,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H85" t="n">
+        <v>45.56861</v>
+      </c>
+      <c r="I85" t="n">
+        <v>-73.66397000000001</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3258,6 +3773,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H86" t="n">
+        <v>45.55674</v>
+      </c>
+      <c r="I86" t="n">
+        <v>-73.67189</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3291,6 +3812,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H87" t="n">
+        <v>45.496</v>
+      </c>
+      <c r="I87" t="n">
+        <v>-73.69867000000001</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3324,6 +3851,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H88" t="n">
+        <v>45.55636</v>
+      </c>
+      <c r="I88" t="n">
+        <v>-73.67305</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3357,6 +3890,12 @@
           <t>Saint-Laurent</t>
         </is>
       </c>
+      <c r="H89" t="n">
+        <v>45.49281</v>
+      </c>
+      <c r="I89" t="n">
+        <v>-73.69902999999999</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3390,6 +3929,12 @@
           <t>Ahuntsic</t>
         </is>
       </c>
+      <c r="H90" t="n">
+        <v>45.56914</v>
+      </c>
+      <c r="I90" t="n">
+        <v>-73.67961</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3423,6 +3968,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H91" t="n">
+        <v>45.6039</v>
+      </c>
+      <c r="I91" t="n">
+        <v>-73.70775999999999</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3456,6 +4007,12 @@
           <t>Outremont</t>
         </is>
       </c>
+      <c r="H92" t="n">
+        <v>45.52518</v>
+      </c>
+      <c r="I92" t="n">
+        <v>-73.6139</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3489,6 +4046,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H93" t="n">
+        <v>45.46502</v>
+      </c>
+      <c r="I93" t="n">
+        <v>-73.8537</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3522,6 +4085,12 @@
           <t>Downtown Montreal</t>
         </is>
       </c>
+      <c r="H94" t="n">
+        <v>45.49643</v>
+      </c>
+      <c r="I94" t="n">
+        <v>-73.58062</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3555,6 +4124,12 @@
           <t>Laval</t>
         </is>
       </c>
+      <c r="H95" t="n">
+        <v>45.59397</v>
+      </c>
+      <c r="I95" t="n">
+        <v>-73.70126999999999</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3588,6 +4163,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H96" t="n">
+        <v>45.45511</v>
+      </c>
+      <c r="I96" t="n">
+        <v>-73.84913</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3621,6 +4202,12 @@
           <t>West Island</t>
         </is>
       </c>
+      <c r="H97" t="n">
+        <v>45.45427</v>
+      </c>
+      <c r="I97" t="n">
+        <v>-73.86337</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3654,6 +4241,12 @@
           <t>Verdun</t>
         </is>
       </c>
+      <c r="H98" t="n">
+        <v>45.46164</v>
+      </c>
+      <c r="I98" t="n">
+        <v>-73.55262</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3687,6 +4280,12 @@
           <t>LaSalle</t>
         </is>
       </c>
+      <c r="H99" t="n">
+        <v>45.43736</v>
+      </c>
+      <c r="I99" t="n">
+        <v>-73.62300999999999</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3720,6 +4319,12 @@
           <t>Hochelaga</t>
         </is>
       </c>
+      <c r="H100" t="n">
+        <v>45.55252</v>
+      </c>
+      <c r="I100" t="n">
+        <v>-73.53757</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3752,6 +4357,12 @@
         <is>
           <t>Verdun</t>
         </is>
+      </c>
+      <c r="H101" t="n">
+        <v>45.46637</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-73.5797</v>
       </c>
     </row>
   </sheetData>
@@ -6228,4 +6839,420 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Place ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Location Area</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SP-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Montreal Convention Centre Emergency Shelter</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1001 Place Jean-Paul-Riopelle, Montreal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Downtown Montreal</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>45.5055</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-73.56100000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>500</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Emergency Shelter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SP-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Olympic Stadium Evacuation Centre</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4545 Pierre-de-Coubertin Ave, Montreal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hochelaga</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>45.5579</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-73.5517</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Mega Shelter</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SP-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Centre Claude-Robillard Community Hub</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1000 Emery St, Montreal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ahuntsic</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>45.547</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-73.652</v>
+      </c>
+      <c r="G4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Community Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SP-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Laval Emergency Reception Centre</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1300 Laval Blvd, Laval</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Laval</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>45.606</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-73.712</v>
+      </c>
+      <c r="G5" t="n">
+        <v>400</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Emergency Shelter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SP-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Longueuil Civic Centre Safe Zone</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1500 De Gentilly Blvd, Longueuil</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Longueuil</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>45.531</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-73.518</v>
+      </c>
+      <c r="G6" t="n">
+        <v>350</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Civic Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SP-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Saint-Laurent Community Shelter</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>8255 Ave Marcel-Laurin, Saint-Laurent</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Saint-Laurent</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>45.508</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-73.69499999999999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>250</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Community Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SP-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>West Island Emergency Reception</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>200 Blvd St-Jean, Pointe-Claire</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>West Island</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>45.448</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-73.815</v>
+      </c>
+      <c r="G8" t="n">
+        <v>300</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Emergency Shelter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SP-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Verdun Recreation Centre Safe Point</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5955 Bannantyne Ave, Verdun</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Verdun</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>45.458</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-73.571</v>
+      </c>
+      <c r="G9" t="n">
+        <v>200</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Recreation Centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SP-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Outremont High-Ground Assembly Point</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>999 Ave Bloomfield, Outremont</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Outremont</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>45.522</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-73.61</v>
+      </c>
+      <c r="G10" t="n">
+        <v>150</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Assembly Point</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SP-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NDG Community Safe Haven</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4333 Cote-St-Antoine Rd, Montreal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NDG</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>45.481</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-73.598</v>
+      </c>
+      <c r="G11" t="n">
+        <v>220</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Community Centre</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>